<commit_message>
chore: qn2 task done
</commit_message>
<xml_diff>
--- a/into-to-python/task-1/stdsscores.xlsx
+++ b/into-to-python/task-1/stdsscores.xlsx
@@ -10,7 +10,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="oUhVWy/i16SWn//ifV2p7TiGwQo5Rx06G3XSESoL9go="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="ZNr+LTNzKWuf1yG6XjK/ZLXzXQ5Dm7W34NZ5Hyv5byQ="/>
     </ext>
   </extLst>
 </workbook>
@@ -33682,7 +33682,7 @@
         <v>41</v>
       </c>
       <c r="F2" s="3">
-        <f t="shared" ref="F2:F9" si="2">ROUND(E2:E251*0.5 + D2:D251*0.5, 1)</f>
+        <f t="shared" ref="F2:F3" si="2">ROUND(E2:E251*0.5 + D2:D251*0.5, 1)</f>
         <v>61.4</v>
       </c>
       <c r="G2" s="3" t="str">
@@ -33786,7 +33786,7 @@
         <v>63</v>
       </c>
       <c r="F4" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="F4:F9" si="5">ROUND(E4:E254*0.5 + D4:D254*0.5, 1)</f>
         <v>66.8</v>
       </c>
       <c r="G4" s="3" t="str">
@@ -33834,7 +33834,7 @@
         <v>23</v>
       </c>
       <c r="F5" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>29.9</v>
       </c>
       <c r="G5" s="3" t="str">
@@ -33882,7 +33882,7 @@
         <v>35</v>
       </c>
       <c r="F6" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>65.7</v>
       </c>
       <c r="G6" s="3" t="str">
@@ -33930,7 +33930,7 @@
         <v>46</v>
       </c>
       <c r="F7" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>63.2</v>
       </c>
       <c r="G7" s="3" t="str">
@@ -33978,7 +33978,7 @@
         <v>57</v>
       </c>
       <c r="F8" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>67.4</v>
       </c>
       <c r="G8" s="3" t="str">
@@ -34026,7 +34026,7 @@
         <v>76</v>
       </c>
       <c r="F9" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>73.7</v>
       </c>
       <c r="G9" s="3" t="str">
@@ -34074,7 +34074,7 @@
         <v>55</v>
       </c>
       <c r="F10" s="3">
-        <f t="shared" ref="F10:F251" si="5">ROUND(E10:E260*0.5 + D10:D260*0.5, 1)</f>
+        <f t="shared" ref="F10:F251" si="6">ROUND(E10:E261*0.5 + D10:D261*0.5, 1)</f>
         <v>43</v>
       </c>
       <c r="G10" s="3" t="str">
@@ -34122,7 +34122,7 @@
         <v>77</v>
       </c>
       <c r="F11" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.1</v>
       </c>
       <c r="G11" s="3" t="str">
@@ -34170,7 +34170,7 @@
         <v>81</v>
       </c>
       <c r="F12" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>87.2</v>
       </c>
       <c r="G12" s="3" t="str">
@@ -34218,7 +34218,7 @@
         <v>66</v>
       </c>
       <c r="F13" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>65</v>
       </c>
       <c r="G13" s="3" t="str">
@@ -34266,7 +34266,7 @@
         <v>13</v>
       </c>
       <c r="F14" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>47.8</v>
       </c>
       <c r="G14" s="3" t="str">
@@ -34314,7 +34314,7 @@
         <v>47</v>
       </c>
       <c r="F15" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>73</v>
       </c>
       <c r="G15" s="3" t="str">
@@ -34362,7 +34362,7 @@
         <v>66</v>
       </c>
       <c r="F16" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>72.3</v>
       </c>
       <c r="G16" s="3" t="str">
@@ -34410,7 +34410,7 @@
         <v>66</v>
       </c>
       <c r="F17" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>81.2</v>
       </c>
       <c r="G17" s="3" t="str">
@@ -34458,7 +34458,7 @@
         <v>32</v>
       </c>
       <c r="F18" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>44.3</v>
       </c>
       <c r="G18" s="3" t="str">
@@ -34506,7 +34506,7 @@
         <v>89</v>
       </c>
       <c r="F19" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>52.4</v>
       </c>
       <c r="G19" s="3" t="str">
@@ -34554,7 +34554,7 @@
         <v>40</v>
       </c>
       <c r="F20" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>56.1</v>
       </c>
       <c r="G20" s="3" t="str">
@@ -34602,7 +34602,7 @@
         <v>89</v>
       </c>
       <c r="F21" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>68</v>
       </c>
       <c r="G21" s="3" t="str">
@@ -34650,7 +34650,7 @@
         <v>85</v>
       </c>
       <c r="F22" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>69.4</v>
       </c>
       <c r="G22" s="3" t="str">
@@ -34698,7 +34698,7 @@
         <v>59</v>
       </c>
       <c r="F23" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>63.7</v>
       </c>
       <c r="G23" s="3" t="str">
@@ -34746,7 +34746,7 @@
         <v>19</v>
       </c>
       <c r="F24" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>36.9</v>
       </c>
       <c r="G24" s="3" t="str">
@@ -34794,7 +34794,7 @@
         <v>37</v>
       </c>
       <c r="F25" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>43.3</v>
       </c>
       <c r="G25" s="3" t="str">
@@ -34842,7 +34842,7 @@
         <v>19</v>
       </c>
       <c r="F26" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>36.4</v>
       </c>
       <c r="G26" s="3" t="str">
@@ -34890,7 +34890,7 @@
         <v>72</v>
       </c>
       <c r="F27" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>70.8</v>
       </c>
       <c r="G27" s="3" t="str">
@@ -34938,7 +34938,7 @@
         <v>27</v>
       </c>
       <c r="F28" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>37.9</v>
       </c>
       <c r="G28" s="3" t="str">
@@ -34986,7 +34986,7 @@
         <v>23</v>
       </c>
       <c r="F29" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>47.1</v>
       </c>
       <c r="G29" s="3" t="str">
@@ -35034,7 +35034,7 @@
         <v>79</v>
       </c>
       <c r="F30" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>58</v>
       </c>
       <c r="G30" s="3" t="str">
@@ -35082,7 +35082,7 @@
         <v>59</v>
       </c>
       <c r="F31" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>49.8</v>
       </c>
       <c r="G31" s="3" t="str">
@@ -35130,7 +35130,7 @@
         <v>74</v>
       </c>
       <c r="F32" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>48.5</v>
       </c>
       <c r="G32" s="3" t="str">
@@ -35178,7 +35178,7 @@
         <v>57</v>
       </c>
       <c r="F33" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>33.6</v>
       </c>
       <c r="G33" s="3" t="str">
@@ -35226,7 +35226,7 @@
         <v>36</v>
       </c>
       <c r="F34" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>37.8</v>
       </c>
       <c r="G34" s="3" t="str">
@@ -35274,7 +35274,7 @@
         <v>33</v>
       </c>
       <c r="F35" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>54.6</v>
       </c>
       <c r="G35" s="3" t="str">
@@ -35322,7 +35322,7 @@
         <v>59</v>
       </c>
       <c r="F36" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>45</v>
       </c>
       <c r="G36" s="3" t="str">
@@ -35370,7 +35370,7 @@
         <v>51</v>
       </c>
       <c r="F37" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.5</v>
       </c>
       <c r="G37" s="3" t="str">
@@ -35418,7 +35418,7 @@
         <v>45</v>
       </c>
       <c r="F38" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>33.5</v>
       </c>
       <c r="G38" s="3" t="str">
@@ -35466,7 +35466,7 @@
         <v>64</v>
       </c>
       <c r="F39" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>38</v>
       </c>
       <c r="G39" s="3" t="str">
@@ -35514,7 +35514,7 @@
         <v>71</v>
       </c>
       <c r="F40" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>85.3</v>
       </c>
       <c r="G40" s="3" t="str">
@@ -35562,7 +35562,7 @@
         <v>46</v>
       </c>
       <c r="F41" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>40.4</v>
       </c>
       <c r="G41" s="3" t="str">
@@ -35610,7 +35610,7 @@
         <v>26</v>
       </c>
       <c r="F42" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>18.8</v>
       </c>
       <c r="G42" s="3" t="str">
@@ -35658,7 +35658,7 @@
         <v>36</v>
       </c>
       <c r="F43" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>62.4</v>
       </c>
       <c r="G43" s="3" t="str">
@@ -35706,7 +35706,7 @@
         <v>49</v>
       </c>
       <c r="F44" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>60.1</v>
       </c>
       <c r="G44" s="3" t="str">
@@ -35754,7 +35754,7 @@
         <v>54</v>
       </c>
       <c r="F45" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>41.3</v>
       </c>
       <c r="G45" s="3" t="str">
@@ -35802,7 +35802,7 @@
         <v>57</v>
       </c>
       <c r="F46" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>61.2</v>
       </c>
       <c r="G46" s="3" t="str">
@@ -35850,7 +35850,7 @@
         <v>42</v>
       </c>
       <c r="F47" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>65.6</v>
       </c>
       <c r="G47" s="3" t="str">
@@ -35898,7 +35898,7 @@
         <v>44</v>
       </c>
       <c r="F48" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>33.1</v>
       </c>
       <c r="G48" s="3" t="str">
@@ -35946,7 +35946,7 @@
         <v>42</v>
       </c>
       <c r="F49" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>40.1</v>
       </c>
       <c r="G49" s="3" t="str">
@@ -35994,7 +35994,7 @@
         <v>73</v>
       </c>
       <c r="F50" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>66</v>
       </c>
       <c r="G50" s="3" t="str">
@@ -36042,7 +36042,7 @@
         <v>74</v>
       </c>
       <c r="F51" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.7</v>
       </c>
       <c r="G51" s="3" t="str">
@@ -36090,7 +36090,7 @@
         <v>59</v>
       </c>
       <c r="F52" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>45.1</v>
       </c>
       <c r="G52" s="3" t="str">
@@ -36138,7 +36138,7 @@
         <v>53</v>
       </c>
       <c r="F53" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>47.8</v>
       </c>
       <c r="G53" s="3" t="str">
@@ -36186,7 +36186,7 @@
         <v>39</v>
       </c>
       <c r="F54" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>27.1</v>
       </c>
       <c r="G54" s="3" t="str">
@@ -36234,7 +36234,7 @@
         <v>43</v>
       </c>
       <c r="F55" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>50.3</v>
       </c>
       <c r="G55" s="3" t="str">
@@ -36282,7 +36282,7 @@
         <v>44</v>
       </c>
       <c r="F56" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>65.4</v>
       </c>
       <c r="G56" s="3" t="str">
@@ -36330,7 +36330,7 @@
         <v>49</v>
       </c>
       <c r="F57" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.8</v>
       </c>
       <c r="G57" s="3" t="str">
@@ -36378,7 +36378,7 @@
         <v>58</v>
       </c>
       <c r="F58" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>57.6</v>
       </c>
       <c r="G58" s="3" t="str">
@@ -36426,7 +36426,7 @@
         <v>63</v>
       </c>
       <c r="F59" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>69.5</v>
       </c>
       <c r="G59" s="3" t="str">
@@ -36474,7 +36474,7 @@
         <v>51</v>
       </c>
       <c r="F60" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>52.2</v>
       </c>
       <c r="G60" s="3" t="str">
@@ -36522,7 +36522,7 @@
         <v>74</v>
       </c>
       <c r="F61" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>56.6</v>
       </c>
       <c r="G61" s="3" t="str">
@@ -36570,7 +36570,7 @@
         <v>61</v>
       </c>
       <c r="F62" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>52.7</v>
       </c>
       <c r="G62" s="3" t="str">
@@ -36618,7 +36618,7 @@
         <v>66</v>
       </c>
       <c r="F63" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>76.6</v>
       </c>
       <c r="G63" s="3" t="str">
@@ -36666,7 +36666,7 @@
         <v>59</v>
       </c>
       <c r="F64" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>78.2</v>
       </c>
       <c r="G64" s="3" t="str">
@@ -36714,7 +36714,7 @@
         <v>49</v>
       </c>
       <c r="F65" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>63.8</v>
       </c>
       <c r="G65" s="3" t="str">
@@ -36762,7 +36762,7 @@
         <v>59</v>
       </c>
       <c r="F66" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>66.8</v>
       </c>
       <c r="G66" s="3" t="str">
@@ -36810,7 +36810,7 @@
         <v>34</v>
       </c>
       <c r="F67" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>28.8</v>
       </c>
       <c r="G67" s="3" t="str">
@@ -36858,7 +36858,7 @@
         <v>54</v>
       </c>
       <c r="F68" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>48.6</v>
       </c>
       <c r="G68" s="3" t="str">
@@ -36906,7 +36906,7 @@
         <v>64</v>
       </c>
       <c r="F69" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>37.8</v>
       </c>
       <c r="G69" s="3" t="str">
@@ -36954,7 +36954,7 @@
         <v>57</v>
       </c>
       <c r="F70" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>54.3</v>
       </c>
       <c r="G70" s="3" t="str">
@@ -37002,7 +37002,7 @@
         <v>61</v>
       </c>
       <c r="F71" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>40</v>
       </c>
       <c r="G71" s="3" t="str">
@@ -37050,7 +37050,7 @@
         <v>61</v>
       </c>
       <c r="F72" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>60.2</v>
       </c>
       <c r="G72" s="3" t="str">
@@ -37098,7 +37098,7 @@
         <v>64</v>
       </c>
       <c r="F73" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.9</v>
       </c>
       <c r="G73" s="3" t="str">
@@ -37146,7 +37146,7 @@
         <v>68</v>
       </c>
       <c r="F74" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>68.5</v>
       </c>
       <c r="G74" s="3" t="str">
@@ -37194,7 +37194,7 @@
         <v>53</v>
       </c>
       <c r="F75" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>34.3</v>
       </c>
       <c r="G75" s="3" t="str">
@@ -37242,7 +37242,7 @@
         <v>68</v>
       </c>
       <c r="F76" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>72.7</v>
       </c>
       <c r="G76" s="3" t="str">
@@ -37290,7 +37290,7 @@
         <v>85</v>
       </c>
       <c r="F77" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>58.7</v>
       </c>
       <c r="G77" s="3" t="str">
@@ -37338,7 +37338,7 @@
         <v>69</v>
       </c>
       <c r="F78" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>73.7</v>
       </c>
       <c r="G78" s="3" t="str">
@@ -37386,7 +37386,7 @@
         <v>34</v>
       </c>
       <c r="F79" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>54.6</v>
       </c>
       <c r="G79" s="3" t="str">
@@ -37434,7 +37434,7 @@
         <v>43</v>
       </c>
       <c r="F80" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>69.8</v>
       </c>
       <c r="G80" s="3" t="str">
@@ -37482,7 +37482,7 @@
         <v>37</v>
       </c>
       <c r="F81" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>64</v>
       </c>
       <c r="G81" s="3" t="str">
@@ -37530,7 +37530,7 @@
         <v>29</v>
       </c>
       <c r="F82" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.9</v>
       </c>
       <c r="G82" s="3" t="str">
@@ -37578,7 +37578,7 @@
         <v>38</v>
       </c>
       <c r="F83" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>48.3</v>
       </c>
       <c r="G83" s="3" t="str">
@@ -37626,7 +37626,7 @@
         <v>69</v>
       </c>
       <c r="F84" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>49.5</v>
       </c>
       <c r="G84" s="3" t="str">
@@ -37674,7 +37674,7 @@
         <v>47</v>
       </c>
       <c r="F85" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>46.1</v>
       </c>
       <c r="G85" s="3" t="str">
@@ -37722,7 +37722,7 @@
         <v>43</v>
       </c>
       <c r="F86" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>44.2</v>
       </c>
       <c r="G86" s="3" t="str">
@@ -37770,7 +37770,7 @@
         <v>35</v>
       </c>
       <c r="F87" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>53.7</v>
       </c>
       <c r="G87" s="3" t="str">
@@ -37818,7 +37818,7 @@
         <v>45</v>
       </c>
       <c r="F88" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>31.5</v>
       </c>
       <c r="G88" s="3" t="str">
@@ -37866,7 +37866,7 @@
         <v>14</v>
       </c>
       <c r="F89" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.2</v>
       </c>
       <c r="G89" s="3" t="str">
@@ -37914,7 +37914,7 @@
         <v>48</v>
       </c>
       <c r="F90" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>49.8</v>
       </c>
       <c r="G90" s="3" t="str">
@@ -37962,7 +37962,7 @@
         <v>70</v>
       </c>
       <c r="F91" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>65.3</v>
       </c>
       <c r="G91" s="3" t="str">
@@ -38010,7 +38010,7 @@
         <v>16</v>
       </c>
       <c r="F92" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>50.9</v>
       </c>
       <c r="G92" s="3" t="str">
@@ -38058,7 +38058,7 @@
         <v>57</v>
       </c>
       <c r="F93" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>45.6</v>
       </c>
       <c r="G93" s="3" t="str">
@@ -38106,7 +38106,7 @@
         <v>28</v>
       </c>
       <c r="F94" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>26.1</v>
       </c>
       <c r="G94" s="3" t="str">
@@ -38154,7 +38154,7 @@
         <v>47</v>
       </c>
       <c r="F95" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>58.1</v>
       </c>
       <c r="G95" s="3" t="str">
@@ -38202,7 +38202,7 @@
         <v>23</v>
       </c>
       <c r="F96" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>37.8</v>
       </c>
       <c r="G96" s="3" t="str">
@@ -38250,7 +38250,7 @@
         <v>51</v>
       </c>
       <c r="F97" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>61.8</v>
       </c>
       <c r="G97" s="3" t="str">
@@ -38298,7 +38298,7 @@
         <v>56</v>
       </c>
       <c r="F98" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>39.6</v>
       </c>
       <c r="G98" s="3" t="str">
@@ -38346,7 +38346,7 @@
         <v>28</v>
       </c>
       <c r="F99" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>32</v>
       </c>
       <c r="G99" s="3" t="str">
@@ -38394,7 +38394,7 @@
         <v>95</v>
       </c>
       <c r="F100" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>85.2</v>
       </c>
       <c r="G100" s="3" t="str">
@@ -38442,7 +38442,7 @@
         <v>71</v>
       </c>
       <c r="F101" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>58.8</v>
       </c>
       <c r="G101" s="3" t="str">
@@ -38490,7 +38490,7 @@
         <v>28</v>
       </c>
       <c r="F102" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>36.3</v>
       </c>
       <c r="G102" s="3" t="str">
@@ -38538,7 +38538,7 @@
         <v>75</v>
       </c>
       <c r="F103" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.1</v>
       </c>
       <c r="G103" s="3" t="str">
@@ -38586,7 +38586,7 @@
         <v>44</v>
       </c>
       <c r="F104" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>28</v>
       </c>
       <c r="G104" s="3" t="str">
@@ -38634,7 +38634,7 @@
         <v>73</v>
       </c>
       <c r="F105" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>66.2</v>
       </c>
       <c r="G105" s="3" t="str">
@@ -38682,7 +38682,7 @@
         <v>37</v>
       </c>
       <c r="F106" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>68.3</v>
       </c>
       <c r="G106" s="3" t="str">
@@ -38730,7 +38730,7 @@
         <v>31</v>
       </c>
       <c r="F107" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.7</v>
       </c>
       <c r="G107" s="3" t="str">
@@ -38778,7 +38778,7 @@
         <v>46</v>
       </c>
       <c r="F108" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>68.3</v>
       </c>
       <c r="G108" s="3" t="str">
@@ -38826,7 +38826,7 @@
         <v>43</v>
       </c>
       <c r="F109" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>60.9</v>
       </c>
       <c r="G109" s="3" t="str">
@@ -38874,7 +38874,7 @@
         <v>53</v>
       </c>
       <c r="F110" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>44.2</v>
       </c>
       <c r="G110" s="3" t="str">
@@ -38922,7 +38922,7 @@
         <v>52</v>
       </c>
       <c r="F111" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>37.9</v>
       </c>
       <c r="G111" s="3" t="str">
@@ -38970,7 +38970,7 @@
         <v>71</v>
       </c>
       <c r="F112" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>65.4</v>
       </c>
       <c r="G112" s="3" t="str">
@@ -39018,7 +39018,7 @@
         <v>57</v>
       </c>
       <c r="F113" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>71.8</v>
       </c>
       <c r="G113" s="3" t="str">
@@ -39066,7 +39066,7 @@
         <v>81</v>
       </c>
       <c r="F114" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>89.4</v>
       </c>
       <c r="G114" s="3" t="str">
@@ -39114,7 +39114,7 @@
         <v>41</v>
       </c>
       <c r="F115" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>59</v>
       </c>
       <c r="G115" s="3" t="str">
@@ -39162,7 +39162,7 @@
         <v>54</v>
       </c>
       <c r="F116" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>76.7</v>
       </c>
       <c r="G116" s="3" t="str">
@@ -39210,7 +39210,7 @@
         <v>70</v>
       </c>
       <c r="F117" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>69.3</v>
       </c>
       <c r="G117" s="3" t="str">
@@ -39258,7 +39258,7 @@
         <v>70</v>
       </c>
       <c r="F118" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>46</v>
       </c>
       <c r="G118" s="3" t="str">
@@ -39306,7 +39306,7 @@
         <v>28</v>
       </c>
       <c r="F119" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>60.9</v>
       </c>
       <c r="G119" s="3" t="str">
@@ -39354,7 +39354,7 @@
         <v>76</v>
       </c>
       <c r="F120" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>83.5</v>
       </c>
       <c r="G120" s="3" t="str">
@@ -39402,7 +39402,7 @@
         <v>22</v>
       </c>
       <c r="F121" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>48.8</v>
       </c>
       <c r="G121" s="3" t="str">
@@ -39450,7 +39450,7 @@
         <v>59</v>
       </c>
       <c r="F122" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>42.4</v>
       </c>
       <c r="G122" s="3" t="str">
@@ -39498,7 +39498,7 @@
         <v>68</v>
       </c>
       <c r="F123" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>58.2</v>
       </c>
       <c r="G123" s="3" t="str">
@@ -39546,7 +39546,7 @@
         <v>43</v>
       </c>
       <c r="F124" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>70.4</v>
       </c>
       <c r="G124" s="3" t="str">
@@ -39594,7 +39594,7 @@
         <v>70</v>
       </c>
       <c r="F125" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>84.9</v>
       </c>
       <c r="G125" s="3" t="str">
@@ -39642,7 +39642,7 @@
         <v>78</v>
       </c>
       <c r="F126" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>59.5</v>
       </c>
       <c r="G126" s="3" t="str">
@@ -39690,7 +39690,7 @@
         <v>55</v>
       </c>
       <c r="F127" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>41.3</v>
       </c>
       <c r="G127" s="3" t="str">
@@ -39738,7 +39738,7 @@
         <v>37</v>
       </c>
       <c r="F128" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>26.7</v>
       </c>
       <c r="G128" s="3" t="str">
@@ -39786,7 +39786,7 @@
         <v>33</v>
       </c>
       <c r="F129" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.7</v>
       </c>
       <c r="G129" s="3" t="str">
@@ -39834,7 +39834,7 @@
         <v>45</v>
       </c>
       <c r="F130" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>34.1</v>
       </c>
       <c r="G130" s="3" t="str">
@@ -39882,7 +39882,7 @@
         <v>71</v>
       </c>
       <c r="F131" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>41.6</v>
       </c>
       <c r="G131" s="3" t="str">
@@ -39930,7 +39930,7 @@
         <v>40</v>
       </c>
       <c r="F132" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>33.2</v>
       </c>
       <c r="G132" s="3" t="str">
@@ -39978,7 +39978,7 @@
         <v>39</v>
       </c>
       <c r="F133" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>65.5</v>
       </c>
       <c r="G133" s="3" t="str">
@@ -40026,7 +40026,7 @@
         <v>47</v>
       </c>
       <c r="F134" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>62.4</v>
       </c>
       <c r="G134" s="3" t="str">
@@ -40074,7 +40074,7 @@
         <v>61</v>
       </c>
       <c r="F135" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>46.2</v>
       </c>
       <c r="G135" s="3" t="str">
@@ -40122,7 +40122,7 @@
         <v>53</v>
       </c>
       <c r="F136" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>38.7</v>
       </c>
       <c r="G136" s="3" t="str">
@@ -40170,7 +40170,7 @@
         <v>34</v>
       </c>
       <c r="F137" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>23.6</v>
       </c>
       <c r="G137" s="3" t="str">
@@ -40218,7 +40218,7 @@
         <v>67</v>
       </c>
       <c r="F138" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>64</v>
       </c>
       <c r="G138" s="3" t="str">
@@ -40266,7 +40266,7 @@
         <v>40</v>
       </c>
       <c r="F139" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>46</v>
       </c>
       <c r="G139" s="3" t="str">
@@ -40314,7 +40314,7 @@
         <v>51</v>
       </c>
       <c r="F140" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.6</v>
       </c>
       <c r="G140" s="3" t="str">
@@ -40362,7 +40362,7 @@
         <v>56</v>
       </c>
       <c r="F141" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>42.3</v>
       </c>
       <c r="G141" s="3" t="str">
@@ -40410,7 +40410,7 @@
         <v>70</v>
       </c>
       <c r="F142" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.8</v>
       </c>
       <c r="G142" s="3" t="str">
@@ -40458,7 +40458,7 @@
         <v>53</v>
       </c>
       <c r="F143" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>33.1</v>
       </c>
       <c r="G143" s="3" t="str">
@@ -40506,7 +40506,7 @@
         <v>70</v>
       </c>
       <c r="F144" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>68.4</v>
       </c>
       <c r="G144" s="3" t="str">
@@ -40554,7 +40554,7 @@
         <v>46</v>
       </c>
       <c r="F145" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>41.1</v>
       </c>
       <c r="G145" s="3" t="str">
@@ -40602,7 +40602,7 @@
         <v>35</v>
       </c>
       <c r="F146" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>22.6</v>
       </c>
       <c r="G146" s="3" t="str">
@@ -40650,7 +40650,7 @@
         <v>71</v>
       </c>
       <c r="F147" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>84.8</v>
       </c>
       <c r="G147" s="3" t="str">
@@ -40698,7 +40698,7 @@
         <v>76</v>
       </c>
       <c r="F148" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>71.8</v>
       </c>
       <c r="G148" s="3" t="str">
@@ -40746,7 +40746,7 @@
         <v>51</v>
       </c>
       <c r="F149" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>62.8</v>
       </c>
       <c r="G149" s="3" t="str">
@@ -40794,7 +40794,7 @@
         <v>63</v>
       </c>
       <c r="F150" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>41.3</v>
       </c>
       <c r="G150" s="3" t="str">
@@ -40842,7 +40842,7 @@
         <v>56</v>
       </c>
       <c r="F151" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>39.6</v>
       </c>
       <c r="G151" s="3" t="str">
@@ -40890,7 +40890,7 @@
         <v>37</v>
       </c>
       <c r="F152" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>27.5</v>
       </c>
       <c r="G152" s="3" t="str">
@@ -40938,7 +40938,7 @@
         <v>42</v>
       </c>
       <c r="F153" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>39.7</v>
       </c>
       <c r="G153" s="3" t="str">
@@ -40986,7 +40986,7 @@
         <v>33</v>
       </c>
       <c r="F154" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>64.9</v>
       </c>
       <c r="G154" s="3" t="str">
@@ -41034,7 +41034,7 @@
         <v>82</v>
       </c>
       <c r="F155" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>82</v>
       </c>
       <c r="G155" s="3" t="str">
@@ -41082,7 +41082,7 @@
         <v>51</v>
       </c>
       <c r="F156" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>52.2</v>
       </c>
       <c r="G156" s="3" t="str">
@@ -41130,7 +41130,7 @@
         <v>82</v>
       </c>
       <c r="F157" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>82.7</v>
       </c>
       <c r="G157" s="3" t="str">
@@ -41178,7 +41178,7 @@
         <v>57</v>
       </c>
       <c r="F158" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>72.3</v>
       </c>
       <c r="G158" s="3" t="str">
@@ -41226,7 +41226,7 @@
         <v>66</v>
       </c>
       <c r="F159" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>81.9</v>
       </c>
       <c r="G159" s="3" t="str">
@@ -41274,7 +41274,7 @@
         <v>62</v>
       </c>
       <c r="F160" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>56.6</v>
       </c>
       <c r="G160" s="3" t="str">
@@ -41322,7 +41322,7 @@
         <v>73</v>
       </c>
       <c r="F161" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>63.5</v>
       </c>
       <c r="G161" s="3" t="str">
@@ -41370,7 +41370,7 @@
         <v>88</v>
       </c>
       <c r="F162" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>56.1</v>
       </c>
       <c r="G162" s="3" t="str">
@@ -41418,7 +41418,7 @@
         <v>39</v>
       </c>
       <c r="F163" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>34.4</v>
       </c>
       <c r="G163" s="3" t="str">
@@ -41466,7 +41466,7 @@
         <v>48</v>
       </c>
       <c r="F164" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>54.8</v>
       </c>
       <c r="G164" s="3" t="str">
@@ -41514,7 +41514,7 @@
         <v>36</v>
       </c>
       <c r="F165" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.2</v>
       </c>
       <c r="G165" s="3" t="str">
@@ -41562,7 +41562,7 @@
         <v>53</v>
       </c>
       <c r="F166" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>32.3</v>
       </c>
       <c r="G166" s="3" t="str">
@@ -41610,7 +41610,7 @@
         <v>77</v>
       </c>
       <c r="F167" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>86.8</v>
       </c>
       <c r="G167" s="3" t="str">
@@ -41658,7 +41658,7 @@
         <v>32</v>
       </c>
       <c r="F168" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>42.5</v>
       </c>
       <c r="G168" s="3" t="str">
@@ -41706,7 +41706,7 @@
         <v>59</v>
       </c>
       <c r="F169" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>71.7</v>
       </c>
       <c r="G169" s="3" t="str">
@@ -41754,7 +41754,7 @@
         <v>40</v>
       </c>
       <c r="F170" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51</v>
       </c>
       <c r="G170" s="3" t="str">
@@ -41802,7 +41802,7 @@
         <v>77</v>
       </c>
       <c r="F171" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>74.4</v>
       </c>
       <c r="G171" s="3" t="str">
@@ -41850,7 +41850,7 @@
         <v>60</v>
       </c>
       <c r="F172" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>70.1</v>
       </c>
       <c r="G172" s="3" t="str">
@@ -41898,7 +41898,7 @@
         <v>74</v>
       </c>
       <c r="F173" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>58.7</v>
       </c>
       <c r="G173" s="3" t="str">
@@ -41946,7 +41946,7 @@
         <v>41</v>
       </c>
       <c r="F174" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>62.6</v>
       </c>
       <c r="G174" s="3" t="str">
@@ -41994,7 +41994,7 @@
         <v>85</v>
       </c>
       <c r="F175" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>73.2</v>
       </c>
       <c r="G175" s="3" t="str">
@@ -42042,7 +42042,7 @@
         <v>45</v>
       </c>
       <c r="F176" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>42.4</v>
       </c>
       <c r="G176" s="3" t="str">
@@ -42090,7 +42090,7 @@
         <v>48</v>
       </c>
       <c r="F177" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.9</v>
       </c>
       <c r="G177" s="3" t="str">
@@ -42138,7 +42138,7 @@
         <v>44</v>
       </c>
       <c r="F178" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>60.7</v>
       </c>
       <c r="G178" s="3" t="str">
@@ -42186,7 +42186,7 @@
         <v>44</v>
       </c>
       <c r="F179" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>52.5</v>
       </c>
       <c r="G179" s="3" t="str">
@@ -42234,7 +42234,7 @@
         <v>62</v>
       </c>
       <c r="F180" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>78.2</v>
       </c>
       <c r="G180" s="3" t="str">
@@ -42282,7 +42282,7 @@
         <v>12</v>
       </c>
       <c r="F181" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>28.7</v>
       </c>
       <c r="G181" s="3" t="str">
@@ -42330,7 +42330,7 @@
         <v>54</v>
       </c>
       <c r="F182" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>64.3</v>
       </c>
       <c r="G182" s="3" t="str">
@@ -42378,7 +42378,7 @@
         <v>43</v>
       </c>
       <c r="F183" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.8</v>
       </c>
       <c r="G183" s="3" t="str">
@@ -42426,7 +42426,7 @@
         <v>25</v>
       </c>
       <c r="F184" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>32</v>
       </c>
       <c r="G184" s="3" t="str">
@@ -42474,7 +42474,7 @@
         <v>31</v>
       </c>
       <c r="F185" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>32</v>
       </c>
       <c r="G185" s="3" t="str">
@@ -42522,7 +42522,7 @@
         <v>46</v>
       </c>
       <c r="F186" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>68.4</v>
       </c>
       <c r="G186" s="3" t="str">
@@ -42570,7 +42570,7 @@
         <v>39</v>
       </c>
       <c r="F187" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>41.4</v>
       </c>
       <c r="G187" s="3" t="str">
@@ -42618,7 +42618,7 @@
         <v>47</v>
       </c>
       <c r="F188" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>72.1</v>
       </c>
       <c r="G188" s="3" t="str">
@@ -42666,7 +42666,7 @@
         <v>60</v>
       </c>
       <c r="F189" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>75.8</v>
       </c>
       <c r="G189" s="3" t="str">
@@ -42714,7 +42714,7 @@
         <v>58</v>
       </c>
       <c r="F190" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>49.5</v>
       </c>
       <c r="G190" s="3" t="str">
@@ -42762,7 +42762,7 @@
         <v>76</v>
       </c>
       <c r="F191" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>72.2</v>
       </c>
       <c r="G191" s="3" t="str">
@@ -42810,7 +42810,7 @@
         <v>40</v>
       </c>
       <c r="F192" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>59.6</v>
       </c>
       <c r="G192" s="3" t="str">
@@ -42858,7 +42858,7 @@
         <v>62</v>
       </c>
       <c r="F193" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>57.3</v>
       </c>
       <c r="G193" s="3" t="str">
@@ -42906,7 +42906,7 @@
         <v>15</v>
       </c>
       <c r="F194" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>35.5</v>
       </c>
       <c r="G194" s="3" t="str">
@@ -42954,7 +42954,7 @@
         <v>64</v>
       </c>
       <c r="F195" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>71.2</v>
       </c>
       <c r="G195" s="3" t="str">
@@ -43002,7 +43002,7 @@
         <v>63</v>
       </c>
       <c r="F196" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>42.9</v>
       </c>
       <c r="G196" s="3" t="str">
@@ -43050,7 +43050,7 @@
         <v>63</v>
       </c>
       <c r="F197" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>54.2</v>
       </c>
       <c r="G197" s="3" t="str">
@@ -43098,7 +43098,7 @@
         <v>90</v>
       </c>
       <c r="F198" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>92.9</v>
       </c>
       <c r="G198" s="3" t="str">
@@ -43146,7 +43146,7 @@
         <v>70</v>
       </c>
       <c r="F199" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>60.4</v>
       </c>
       <c r="G199" s="3" t="str">
@@ -43194,7 +43194,7 @@
         <v>50</v>
       </c>
       <c r="F200" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>30.6</v>
       </c>
       <c r="G200" s="3" t="str">
@@ -43242,7 +43242,7 @@
         <v>77</v>
       </c>
       <c r="F201" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>68.8</v>
       </c>
       <c r="G201" s="3" t="str">
@@ -43290,7 +43290,7 @@
         <v>77</v>
       </c>
       <c r="F202" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.8</v>
       </c>
       <c r="G202" s="3" t="str">
@@ -43338,7 +43338,7 @@
         <v>45</v>
       </c>
       <c r="F203" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>68.6</v>
       </c>
       <c r="G203" s="3" t="str">
@@ -43386,7 +43386,7 @@
         <v>63</v>
       </c>
       <c r="F204" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>40.6</v>
       </c>
       <c r="G204" s="3" t="str">
@@ -43434,7 +43434,7 @@
         <v>57</v>
       </c>
       <c r="F205" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.4</v>
       </c>
       <c r="G205" s="3" t="str">
@@ -43482,7 +43482,7 @@
         <v>41</v>
       </c>
       <c r="F206" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>25.6</v>
       </c>
       <c r="G206" s="3" t="str">
@@ -43530,7 +43530,7 @@
         <v>60</v>
       </c>
       <c r="F207" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>78</v>
       </c>
       <c r="G207" s="3" t="str">
@@ -43578,7 +43578,7 @@
         <v>59</v>
       </c>
       <c r="F208" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>67.9</v>
       </c>
       <c r="G208" s="3" t="str">
@@ -43626,7 +43626,7 @@
         <v>77</v>
       </c>
       <c r="F209" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>53.8</v>
       </c>
       <c r="G209" s="3" t="str">
@@ -43674,7 +43674,7 @@
         <v>42</v>
       </c>
       <c r="F210" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.9</v>
       </c>
       <c r="G210" s="3" t="str">
@@ -43722,7 +43722,7 @@
         <v>67</v>
       </c>
       <c r="F211" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>56.4</v>
       </c>
       <c r="G211" s="3" t="str">
@@ -43770,7 +43770,7 @@
         <v>76</v>
       </c>
       <c r="F212" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>76.9</v>
       </c>
       <c r="G212" s="3" t="str">
@@ -43818,7 +43818,7 @@
         <v>68</v>
       </c>
       <c r="F213" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>83.8</v>
       </c>
       <c r="G213" s="3" t="str">
@@ -43866,7 +43866,7 @@
         <v>59</v>
       </c>
       <c r="F214" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>58</v>
       </c>
       <c r="G214" s="3" t="str">
@@ -43914,7 +43914,7 @@
         <v>71</v>
       </c>
       <c r="F215" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>76.8</v>
       </c>
       <c r="G215" s="3" t="str">
@@ -43962,7 +43962,7 @@
         <v>62</v>
       </c>
       <c r="F216" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>54</v>
       </c>
       <c r="G216" s="3" t="str">
@@ -44010,7 +44010,7 @@
         <v>91</v>
       </c>
       <c r="F217" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>64.5</v>
       </c>
       <c r="G217" s="3" t="str">
@@ -44058,7 +44058,7 @@
         <v>62</v>
       </c>
       <c r="F218" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>44.4</v>
       </c>
       <c r="G218" s="3" t="str">
@@ -44106,7 +44106,7 @@
         <v>69</v>
       </c>
       <c r="F219" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>53</v>
       </c>
       <c r="G219" s="3" t="str">
@@ -44154,7 +44154,7 @@
         <v>73</v>
       </c>
       <c r="F220" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.4</v>
       </c>
       <c r="G220" s="3" t="str">
@@ -44202,7 +44202,7 @@
         <v>56</v>
       </c>
       <c r="F221" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>43.9</v>
       </c>
       <c r="G221" s="3" t="str">
@@ -44250,7 +44250,7 @@
         <v>59</v>
       </c>
       <c r="F222" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>74.1</v>
       </c>
       <c r="G222" s="3" t="str">
@@ -44298,7 +44298,7 @@
         <v>47</v>
       </c>
       <c r="F223" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>31.9</v>
       </c>
       <c r="G223" s="3" t="str">
@@ -44346,7 +44346,7 @@
         <v>57</v>
       </c>
       <c r="F224" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>43.6</v>
       </c>
       <c r="G224" s="3" t="str">
@@ -44394,7 +44394,7 @@
         <v>64</v>
       </c>
       <c r="F225" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>59.6</v>
       </c>
       <c r="G225" s="3" t="str">
@@ -44442,7 +44442,7 @@
         <v>88</v>
       </c>
       <c r="F226" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>56.7</v>
       </c>
       <c r="G226" s="3" t="str">
@@ -44490,7 +44490,7 @@
         <v>60</v>
       </c>
       <c r="F227" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.2</v>
       </c>
       <c r="G227" s="3" t="str">
@@ -44538,7 +44538,7 @@
         <v>37</v>
       </c>
       <c r="F228" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>31.5</v>
       </c>
       <c r="G228" s="3" t="str">
@@ -44586,7 +44586,7 @@
         <v>32</v>
       </c>
       <c r="F229" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>56.8</v>
       </c>
       <c r="G229" s="3" t="str">
@@ -44634,7 +44634,7 @@
         <v>93</v>
       </c>
       <c r="F230" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>92</v>
       </c>
       <c r="G230" s="3" t="str">
@@ -44682,7 +44682,7 @@
         <v>57</v>
       </c>
       <c r="F231" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>60.1</v>
       </c>
       <c r="G231" s="3" t="str">
@@ -44730,7 +44730,7 @@
         <v>92</v>
       </c>
       <c r="F232" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51.4</v>
       </c>
       <c r="G232" s="3" t="str">
@@ -44778,7 +44778,7 @@
         <v>55</v>
       </c>
       <c r="F233" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>37.7</v>
       </c>
       <c r="G233" s="3" t="str">
@@ -44826,7 +44826,7 @@
         <v>53</v>
       </c>
       <c r="F234" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>32.4</v>
       </c>
       <c r="G234" s="3" t="str">
@@ -44874,7 +44874,7 @@
         <v>64</v>
       </c>
       <c r="F235" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>73.3</v>
       </c>
       <c r="G235" s="3" t="str">
@@ -44922,7 +44922,7 @@
         <v>69</v>
       </c>
       <c r="F236" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>72.3</v>
       </c>
       <c r="G236" s="3" t="str">
@@ -44970,7 +44970,7 @@
         <v>70</v>
       </c>
       <c r="F237" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>81.5</v>
       </c>
       <c r="G237" s="3" t="str">
@@ -45018,7 +45018,7 @@
         <v>42</v>
       </c>
       <c r="F238" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>35.7</v>
       </c>
       <c r="G238" s="3" t="str">
@@ -45066,7 +45066,7 @@
         <v>45</v>
       </c>
       <c r="F239" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>39.1</v>
       </c>
       <c r="G239" s="3" t="str">
@@ -45114,7 +45114,7 @@
         <v>63</v>
       </c>
       <c r="F240" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>55.5</v>
       </c>
       <c r="G240" s="3" t="str">
@@ -45162,7 +45162,7 @@
         <v>30</v>
       </c>
       <c r="F241" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>26.3</v>
       </c>
       <c r="G241" s="3" t="str">
@@ -45210,7 +45210,7 @@
         <v>81</v>
       </c>
       <c r="F242" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>49</v>
       </c>
       <c r="G242" s="3" t="str">
@@ -45258,7 +45258,7 @@
         <v>54</v>
       </c>
       <c r="F243" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>49.1</v>
       </c>
       <c r="G243" s="3" t="str">
@@ -45306,7 +45306,7 @@
         <v>45</v>
       </c>
       <c r="F244" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>67.9</v>
       </c>
       <c r="G244" s="3" t="str">
@@ -45354,7 +45354,7 @@
         <v>80</v>
       </c>
       <c r="F245" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>75</v>
       </c>
       <c r="G245" s="3" t="str">
@@ -45402,7 +45402,7 @@
         <v>44</v>
       </c>
       <c r="F246" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>56.5</v>
       </c>
       <c r="G246" s="3" t="str">
@@ -45450,7 +45450,7 @@
         <v>38</v>
       </c>
       <c r="F247" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>41.2</v>
       </c>
       <c r="G247" s="3" t="str">
@@ -45498,7 +45498,7 @@
         <v>50</v>
       </c>
       <c r="F248" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>69.4</v>
       </c>
       <c r="G248" s="3" t="str">
@@ -45546,7 +45546,7 @@
         <v>72</v>
       </c>
       <c r="F249" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>85.2</v>
       </c>
       <c r="G249" s="3" t="str">
@@ -45594,7 +45594,7 @@
         <v>59</v>
       </c>
       <c r="F250" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>73</v>
       </c>
       <c r="G250" s="3" t="str">
@@ -45642,7 +45642,7 @@
         <v>56</v>
       </c>
       <c r="F251" s="3">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>75.1</v>
       </c>
       <c r="G251" s="3" t="str">
@@ -45702,9 +45702,7 @@
     </row>
     <row r="253" ht="15.75" customHeight="1">
       <c r="A253" s="2"/>
-      <c r="B253" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="B253" s="2"/>
       <c r="C253" s="2"/>
       <c r="D253" s="2"/>
       <c r="E253" s="2"/>
@@ -45732,23 +45730,15 @@
     </row>
     <row r="254" ht="15.75" customHeight="1">
       <c r="A254" s="2"/>
-      <c r="B254" s="5"/>
-      <c r="C254" s="6"/>
-      <c r="D254" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E254" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="F254" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="G254" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H254" s="7" t="s">
-        <v>5</v>
-      </c>
+      <c r="B254" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C254" s="2"/>
+      <c r="D254" s="2"/>
+      <c r="E254" s="2"/>
+      <c r="F254" s="2"/>
+      <c r="G254" s="2"/>
+      <c r="H254" s="2"/>
       <c r="I254" s="2"/>
       <c r="J254" s="2"/>
       <c r="K254" s="2"/>
@@ -45770,29 +45760,22 @@
     </row>
     <row r="255" ht="15.75" customHeight="1">
       <c r="A255" s="2"/>
-      <c r="B255" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C255" s="3"/>
-      <c r="D255" s="8">
-        <f t="shared" ref="D255:E255" si="6">MIN(B2:B251)</f>
-        <v>10.2</v>
-      </c>
-      <c r="E255" s="8">
-        <f t="shared" si="6"/>
-        <v>10.3</v>
-      </c>
-      <c r="F255" s="8">
-        <f>MIN(E2:E251)</f>
-        <v>12</v>
-      </c>
-      <c r="G255" s="8">
-        <f>MIN(D2:D251)</f>
-        <v>10.1</v>
-      </c>
-      <c r="H255" s="8">
-        <f>MIN(F2:F251)</f>
-        <v>18.8</v>
+      <c r="B255" s="5"/>
+      <c r="C255" s="6"/>
+      <c r="D255" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E255" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="F255" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G255" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H255" s="7" t="s">
+        <v>5</v>
       </c>
       <c r="I255" s="2"/>
       <c r="J255" s="2"/>
@@ -45816,28 +45799,28 @@
     <row r="256" ht="15.75" customHeight="1">
       <c r="A256" s="2"/>
       <c r="B256" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C256" s="3"/>
       <c r="D256" s="8">
-        <f t="shared" ref="D256:E256" si="7">MAX(B2:B251)</f>
-        <v>99.8</v>
+        <f t="shared" ref="D256:E256" si="7">MIN(B2:B251)</f>
+        <v>10.2</v>
       </c>
       <c r="E256" s="8">
         <f t="shared" si="7"/>
-        <v>99.4</v>
+        <v>10.3</v>
       </c>
       <c r="F256" s="8">
-        <f>MAX(E2:E251)</f>
-        <v>95</v>
+        <f>MIN(E2:E251)</f>
+        <v>12</v>
       </c>
       <c r="G256" s="8">
-        <f>MAX(D2:D251)</f>
-        <v>100</v>
+        <f>MIN(D2:D251)</f>
+        <v>10.1</v>
       </c>
       <c r="H256" s="8">
-        <f>MAX(F2:F251)</f>
-        <v>92.9</v>
+        <f>MIN(F2:F251)</f>
+        <v>18.8</v>
       </c>
       <c r="I256" s="2"/>
       <c r="J256" s="2"/>
@@ -45860,29 +45843,29 @@
     </row>
     <row r="257" ht="15.75" customHeight="1">
       <c r="A257" s="2"/>
-      <c r="B257" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C257" s="6"/>
+      <c r="B257" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C257" s="3"/>
       <c r="D257" s="8">
-        <f>AVERAGE(B2:B251)</f>
-        <v>54.1336</v>
+        <f t="shared" ref="D257:E257" si="8">MAX(B2:B251)</f>
+        <v>99.8</v>
       </c>
       <c r="E257" s="8">
-        <f>AVERAGE(C2:D251)</f>
-        <v>55.6038</v>
+        <f t="shared" si="8"/>
+        <v>99.4</v>
       </c>
       <c r="F257" s="8">
-        <f>AVERAGE(E2:E251)</f>
-        <v>54.608</v>
+        <f>MAX(E2:E251)</f>
+        <v>95</v>
       </c>
       <c r="G257" s="8">
-        <f>AVERAGE(D2:D251)</f>
-        <v>56.2512</v>
+        <f>MAX(D2:D251)</f>
+        <v>100</v>
       </c>
       <c r="H257" s="8">
-        <f>AVERAGE(F2:F251)</f>
-        <v>55.4544</v>
+        <f>MAX(F2:F251)</f>
+        <v>92.9</v>
       </c>
       <c r="I257" s="2"/>
       <c r="J257" s="2"/>
@@ -45905,13 +45888,30 @@
     </row>
     <row r="258" ht="15.75" customHeight="1">
       <c r="A258" s="2"/>
-      <c r="B258" s="4"/>
-      <c r="C258" s="2"/>
-      <c r="D258" s="2"/>
-      <c r="E258" s="2"/>
-      <c r="F258" s="2"/>
-      <c r="G258" s="2"/>
-      <c r="H258" s="2"/>
+      <c r="B258" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C258" s="6"/>
+      <c r="D258" s="8">
+        <f>AVERAGE(B2:B251)</f>
+        <v>54.1336</v>
+      </c>
+      <c r="E258" s="8">
+        <f>AVERAGE(C2:D251)</f>
+        <v>55.6038</v>
+      </c>
+      <c r="F258" s="8">
+        <f>AVERAGE(E2:E251)</f>
+        <v>54.608</v>
+      </c>
+      <c r="G258" s="8">
+        <f>AVERAGE(D2:D251)</f>
+        <v>56.2512</v>
+      </c>
+      <c r="H258" s="8">
+        <f>AVERAGE(F2:F251)</f>
+        <v>55.4544</v>
+      </c>
       <c r="I258" s="2"/>
       <c r="J258" s="2"/>
       <c r="K258" s="2"/>
@@ -45933,9 +45933,7 @@
     </row>
     <row r="259" ht="15.75" customHeight="1">
       <c r="A259" s="2"/>
-      <c r="B259" s="10" t="s">
-        <v>12</v>
-      </c>
+      <c r="B259" s="4"/>
       <c r="C259" s="2"/>
       <c r="D259" s="2"/>
       <c r="E259" s="2"/>
@@ -45963,15 +45961,12 @@
     </row>
     <row r="260" ht="15.75" customHeight="1">
       <c r="A260" s="2"/>
-      <c r="B260" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C260" s="3"/>
-      <c r="D260" s="3"/>
-      <c r="E260" s="7">
-        <f>COUNTIF(H2:H251, "P")</f>
-        <v>179</v>
-      </c>
+      <c r="B260" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C260" s="2"/>
+      <c r="D260" s="2"/>
+      <c r="E260" s="2"/>
       <c r="F260" s="2"/>
       <c r="G260" s="2"/>
       <c r="H260" s="2"/>
@@ -45997,13 +45992,13 @@
     <row r="261" ht="15.75" customHeight="1">
       <c r="A261" s="2"/>
       <c r="B261" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C261" s="3"/>
       <c r="D261" s="3"/>
       <c r="E261" s="7">
-        <f>COUNTIF(H2:H251, "F")</f>
-        <v>71</v>
+        <f>COUNTIF(H2:H251, "P")</f>
+        <v>179</v>
       </c>
       <c r="F261" s="2"/>
       <c r="G261" s="2"/>
@@ -46029,10 +46024,15 @@
     </row>
     <row r="262" ht="15.75" customHeight="1">
       <c r="A262" s="2"/>
-      <c r="B262" s="2"/>
-      <c r="C262" s="2"/>
-      <c r="D262" s="2"/>
-      <c r="E262" s="2"/>
+      <c r="B262" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C262" s="3"/>
+      <c r="D262" s="3"/>
+      <c r="E262" s="7">
+        <f>COUNTIF(H2:H251, "F")</f>
+        <v>71</v>
+      </c>
       <c r="F262" s="2"/>
       <c r="G262" s="2"/>
       <c r="H262" s="2"/>
@@ -46057,10 +46057,8 @@
     </row>
     <row r="263" ht="15.75" customHeight="1">
       <c r="A263" s="2"/>
-      <c r="B263" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C263" s="4"/>
+      <c r="B263" s="2"/>
+      <c r="C263" s="2"/>
       <c r="D263" s="2"/>
       <c r="E263" s="2"/>
       <c r="F263" s="2"/>
@@ -46087,29 +46085,17 @@
     </row>
     <row r="264" ht="15.75" customHeight="1">
       <c r="A264" s="2"/>
-      <c r="B264" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C264" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D264" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="E264" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F264" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G264" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H264" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I264" s="11"/>
-      <c r="J264" s="11"/>
+      <c r="B264" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C264" s="4"/>
+      <c r="D264" s="2"/>
+      <c r="E264" s="2"/>
+      <c r="F264" s="2"/>
+      <c r="G264" s="2"/>
+      <c r="H264" s="2"/>
+      <c r="I264" s="2"/>
+      <c r="J264" s="2"/>
       <c r="K264" s="2"/>
       <c r="L264" s="2"/>
       <c r="M264" s="2"/>
@@ -46130,31 +46116,25 @@
     <row r="265" ht="15.75" customHeight="1">
       <c r="A265" s="2"/>
       <c r="B265" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C265" s="7">
-        <f>COUNTIF(G2:G251, "A")</f>
-        <v>49</v>
-      </c>
-      <c r="D265" s="7">
-        <f>COUNTIF(G2:G251, "B+")</f>
-        <v>50</v>
-      </c>
-      <c r="E265" s="7">
-        <f>COUNTIF(G2:G251, "B")</f>
-        <v>60</v>
-      </c>
-      <c r="F265" s="7">
-        <f>COUNTIF(G2:G251, "C")</f>
-        <v>44</v>
-      </c>
-      <c r="G265" s="7">
-        <f>COUNTIF(G2:G251, "D")</f>
+        <v>6</v>
+      </c>
+      <c r="C265" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D265" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H265" s="7">
-        <f>COUNTIF(G2:G251, "E")</f>
-        <v>30</v>
+      <c r="E265" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F265" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G265" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H265" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="I265" s="11"/>
       <c r="J265" s="11"/>
@@ -46177,15 +46157,35 @@
     </row>
     <row r="266" ht="15.75" customHeight="1">
       <c r="A266" s="2"/>
-      <c r="B266" s="2"/>
-      <c r="C266" s="2"/>
-      <c r="D266" s="2"/>
-      <c r="E266" s="2"/>
-      <c r="F266" s="2"/>
-      <c r="G266" s="2"/>
-      <c r="H266" s="2"/>
-      <c r="I266" s="2"/>
-      <c r="J266" s="2"/>
+      <c r="B266" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C266" s="7">
+        <f>COUNTIF(G2:G251, "A")</f>
+        <v>49</v>
+      </c>
+      <c r="D266" s="7">
+        <f>COUNTIF(G2:G251, "B+")</f>
+        <v>50</v>
+      </c>
+      <c r="E266" s="7">
+        <f>COUNTIF(G2:G251, "B")</f>
+        <v>60</v>
+      </c>
+      <c r="F266" s="7">
+        <f>COUNTIF(G2:G251, "C")</f>
+        <v>44</v>
+      </c>
+      <c r="G266" s="7">
+        <f>COUNTIF(G2:G251, "D")</f>
+        <v>17</v>
+      </c>
+      <c r="H266" s="7">
+        <f>COUNTIF(G2:G251, "E")</f>
+        <v>30</v>
+      </c>
+      <c r="I266" s="11"/>
+      <c r="J266" s="11"/>
       <c r="K266" s="2"/>
       <c r="L266" s="2"/>
       <c r="M266" s="2"/>
@@ -66783,10 +66783,38 @@
       <c r="Y1001" s="2"/>
       <c r="Z1001" s="2"/>
     </row>
+    <row r="1002" ht="15.75" customHeight="1">
+      <c r="A1002" s="2"/>
+      <c r="B1002" s="2"/>
+      <c r="C1002" s="2"/>
+      <c r="D1002" s="2"/>
+      <c r="E1002" s="2"/>
+      <c r="F1002" s="2"/>
+      <c r="G1002" s="2"/>
+      <c r="H1002" s="2"/>
+      <c r="I1002" s="2"/>
+      <c r="J1002" s="2"/>
+      <c r="K1002" s="2"/>
+      <c r="L1002" s="2"/>
+      <c r="M1002" s="2"/>
+      <c r="N1002" s="2"/>
+      <c r="O1002" s="2"/>
+      <c r="P1002" s="2"/>
+      <c r="Q1002" s="2"/>
+      <c r="R1002" s="2"/>
+      <c r="S1002" s="2"/>
+      <c r="T1002" s="2"/>
+      <c r="U1002" s="2"/>
+      <c r="V1002" s="2"/>
+      <c r="W1002" s="2"/>
+      <c r="X1002" s="2"/>
+      <c r="Y1002" s="2"/>
+      <c r="Z1002" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B254:C254"/>
-    <mergeCell ref="B257:C257"/>
+    <mergeCell ref="B255:C255"/>
+    <mergeCell ref="B258:C258"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>